<commit_message>
Changes - LV_T2274_T2275_EventExpenseCommonFeatures_VerifyValidationRulesOnEventExpenseSet - 27 Oct 2025
</commit_message>
<xml_diff>
--- a/TestData/LV_T1140_T1141_T1151_T1144_T1146_CompaniesAddNewCompanyWithRecordTypeForCapitalProviderAndOperatingCompany.xlsx
+++ b/TestData/LV_T1140_T1141_T1151_T1144_T1146_CompaniesAddNewCompanyWithRecordTypeForCapitalProviderAndOperatingCompany.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SMittal0207\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BADD367F-5961-4200-A328-AB2507072F33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F891328-B48C-4981-82D1-4691BF00BFA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="2" r:id="rId1"/>
@@ -202,9 +202,6 @@
     <t>Next</t>
   </si>
   <si>
-    <t>Error: Company Name: You must enter a value</t>
-  </si>
-  <si>
     <t>CreateCompanyPage</t>
   </si>
   <si>
@@ -248,6 +245,9 @@
   </si>
   <si>
     <t>ListViewsOptions</t>
+  </si>
+  <si>
+    <t>Company Name</t>
   </si>
 </sst>
 </file>
@@ -584,13 +584,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>43</v>
       </c>
@@ -598,7 +598,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>40</v>
       </c>
@@ -606,12 +606,12 @@
         <v>41</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C3" t="s">
         <v>39</v>
@@ -626,14 +626,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBDC019B-D24C-4D11-B55C-3110A9446A1A}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>45</v>
       </c>
@@ -646,17 +646,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF90D989-9E82-487D-8276-51E2EA9B068E}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>47</v>
       </c>
@@ -669,25 +669,25 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:P3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.88671875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="23" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.6640625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="18" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="21.109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.44140625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="22" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="21.85546875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="21.88671875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="21.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -731,13 +731,13 @@
         <v>26</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -763,7 +763,7 @@
         <v>16</v>
       </c>
       <c r="I2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="J2" t="s">
         <v>18</v>
@@ -778,16 +778,16 @@
         <v>24</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="O2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="P2" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>25</v>
       </c>
@@ -803,14 +803,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="2" width="66.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.6640625" customWidth="1"/>
+    <col min="2" max="2" width="66.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>30</v>
       </c>
@@ -821,7 +821,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -832,7 +832,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>36</v>
       </c>
@@ -843,7 +843,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>25</v>
       </c>
@@ -854,7 +854,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>27</v>
       </c>
@@ -865,7 +865,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>28</v>
       </c>
@@ -876,7 +876,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>29</v>
       </c>
@@ -896,13 +896,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04D1D419-ABFD-421C-B68D-C11399E2BB35}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="31.42578125" customWidth="1"/>
-    <col min="2" max="2" width="44.85546875" customWidth="1"/>
+    <col min="1" max="1" width="31.44140625" customWidth="1"/>
+    <col min="2" max="2" width="44.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>30</v>
       </c>
@@ -913,7 +913,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="90" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -924,7 +924,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>36</v>
       </c>
@@ -935,7 +935,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>25</v>
       </c>
@@ -946,7 +946,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>27</v>
       </c>
@@ -957,7 +957,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>28</v>
       </c>
@@ -968,7 +968,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>29</v>
       </c>
@@ -987,29 +987,29 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F8B8E47-1D86-45C9-83BF-075D8B336916}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>48</v>
       </c>
       <c r="B1" s="1"/>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>51</v>
       </c>
@@ -1022,39 +1022,39 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{034FFB1C-D194-4C70-9A1A-86723ADDEF1B}">
   <dimension ref="A1:A6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="26" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>
@@ -1065,19 +1065,19 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17B7266C-CFE5-4470-B8D5-B5EA6A79ADEA}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="42.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="42.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>52</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Code Merge with Sahil Oct 29 2025
</commit_message>
<xml_diff>
--- a/TestData/LV_T1140_T1141_T1151_T1144_T1146_CompaniesAddNewCompanyWithRecordTypeForCapitalProviderAndOperatingCompany.xlsx
+++ b/TestData/LV_T1140_T1141_T1151_T1144_T1146_CompaniesAddNewCompanyWithRecordTypeForCapitalProviderAndOperatingCompany.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SMittal0207\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BADD367F-5961-4200-A328-AB2507072F33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F891328-B48C-4981-82D1-4691BF00BFA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="2" r:id="rId1"/>
@@ -202,9 +202,6 @@
     <t>Next</t>
   </si>
   <si>
-    <t>Error: Company Name: You must enter a value</t>
-  </si>
-  <si>
     <t>CreateCompanyPage</t>
   </si>
   <si>
@@ -248,6 +245,9 @@
   </si>
   <si>
     <t>ListViewsOptions</t>
+  </si>
+  <si>
+    <t>Company Name</t>
   </si>
 </sst>
 </file>
@@ -584,13 +584,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>43</v>
       </c>
@@ -598,7 +598,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>40</v>
       </c>
@@ -606,12 +606,12 @@
         <v>41</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C3" t="s">
         <v>39</v>
@@ -626,14 +626,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBDC019B-D24C-4D11-B55C-3110A9446A1A}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>45</v>
       </c>
@@ -646,17 +646,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF90D989-9E82-487D-8276-51E2EA9B068E}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>47</v>
       </c>
@@ -669,25 +669,25 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:P3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.88671875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="23" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.6640625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="18" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="21.109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.44140625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="22" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="21.85546875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="21.88671875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="21.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -731,13 +731,13 @@
         <v>26</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -763,7 +763,7 @@
         <v>16</v>
       </c>
       <c r="I2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="J2" t="s">
         <v>18</v>
@@ -778,16 +778,16 @@
         <v>24</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="O2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="P2" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>25</v>
       </c>
@@ -803,14 +803,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="2" width="66.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.6640625" customWidth="1"/>
+    <col min="2" max="2" width="66.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>30</v>
       </c>
@@ -821,7 +821,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -832,7 +832,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>36</v>
       </c>
@@ -843,7 +843,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>25</v>
       </c>
@@ -854,7 +854,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>27</v>
       </c>
@@ -865,7 +865,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>28</v>
       </c>
@@ -876,7 +876,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>29</v>
       </c>
@@ -896,13 +896,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04D1D419-ABFD-421C-B68D-C11399E2BB35}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="31.42578125" customWidth="1"/>
-    <col min="2" max="2" width="44.85546875" customWidth="1"/>
+    <col min="1" max="1" width="31.44140625" customWidth="1"/>
+    <col min="2" max="2" width="44.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>30</v>
       </c>
@@ -913,7 +913,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="90" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -924,7 +924,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>36</v>
       </c>
@@ -935,7 +935,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>25</v>
       </c>
@@ -946,7 +946,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>27</v>
       </c>
@@ -957,7 +957,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>28</v>
       </c>
@@ -968,7 +968,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>29</v>
       </c>
@@ -987,29 +987,29 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F8B8E47-1D86-45C9-83BF-075D8B336916}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>48</v>
       </c>
       <c r="B1" s="1"/>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>51</v>
       </c>
@@ -1022,39 +1022,39 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{034FFB1C-D194-4C70-9A1A-86723ADDEF1B}">
   <dimension ref="A1:A6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="26" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>
@@ -1065,19 +1065,19 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17B7266C-CFE5-4470-B8D5-B5EA6A79ADEA}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="42.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="42.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>52</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>

</xml_diff>